<commit_message>
Deployed a745b0ef9 to revision-date with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/revision-date/catalog_summary.xlsx
+++ b/revision-date/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X284"/>
+  <dimension ref="A1:X300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5561,12 +5561,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5576,7 +5576,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5622,7 +5622,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5632,17 +5632,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5671,12 +5671,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5747,12 +5747,12 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5781,12 +5781,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5852,17 +5852,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/1.715740</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -5891,12 +5891,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5962,17 +5962,17 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>10.21966/1.715740</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V51" t="n">
@@ -6221,12 +6221,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6236,7 +6236,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6292,17 +6292,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6312,7 +6312,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6331,12 +6331,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6402,17 +6402,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -8523,12 +8523,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8538,7 +8538,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8580,16 +8580,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8599,12 +8599,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8633,12 +8633,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8648,7 +8648,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8690,16 +8690,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8709,12 +8709,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8724,7 +8724,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -13147,12 +13147,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13162,7 +13162,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13185,7 +13185,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13204,11 +13204,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13223,12 +13223,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13238,7 +13238,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13246,7 +13246,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13257,12 +13257,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13272,7 +13272,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13295,7 +13295,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13314,11 +13314,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13333,12 +13333,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13348,7 +13348,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13356,7 +13356,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -13477,12 +13477,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13492,7 +13492,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13510,12 +13510,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13534,16 +13534,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13553,12 +13553,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13587,12 +13587,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13602,7 +13602,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13620,12 +13620,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13644,16 +13644,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13663,12 +13663,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -14577,12 +14577,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14592,7 +14592,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14610,7 +14610,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14630,7 +14630,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14638,27 +14638,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14668,7 +14668,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14687,12 +14687,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14702,7 +14702,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14720,7 +14720,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14740,7 +14740,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14748,27 +14748,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V131" t="n">
@@ -15229,9 +15229,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X135" t="n">
-        <v>1</v>
-      </c>
+      <c r="X135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -16113,9 +16111,7 @@
           <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X143" t="n">
-        <v>1</v>
-      </c>
+      <c r="X143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -21627,12 +21623,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>ca-cioos_33a367c1-2706-4301-af99-4455fbe189a0</t>
+          <t>ca-cioos_3efdccb0-08ef-4e90-ac91-72969f94a99a</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -21642,7 +21638,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Cryosphere Snow Surveys Southwest British Columbia - Airborne Coastal Observatory</t>
+          <t>Bute Inlet Geohazard - Topography Surveys - 2023 - Hakai Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -21684,16 +21680,16 @@
         </is>
       </c>
       <c r="N194" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.9, 48.62], [-122.1, 48.62], [-122.1, 50.82], [-126.9, 50.82], [-126.9, 48.62]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.9, 50.53], [-124.2, 50.53], [-124.2, 50.99], [-124.9, 50.99], [-124.9, 50.53]]]}</t>
         </is>
       </c>
       <c r="P194" t="inlineStr">
         <is>
-          <t>[{'max': '2300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2600.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q194" t="inlineStr">
@@ -21703,12 +21699,12 @@
       </c>
       <c r="R194" t="inlineStr">
         <is>
-          <t>10.21966/thq7-0g08</t>
+          <t>10.21966/e4b8-vp48</t>
         </is>
       </c>
       <c r="S194" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRfMcU9I8mMcBH6qiv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRG7xQ84LQrgS4jhie</t>
         </is>
       </c>
       <c r="T194" t="inlineStr">
@@ -21718,15 +21714,15 @@
       </c>
       <c r="U194" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="V194" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W194" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
       <c r="X194" t="inlineStr"/>
@@ -21737,12 +21733,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>ca-cioos_3efdccb0-08ef-4e90-ac91-72969f94a99a</t>
+          <t>ca-cioos_43422dc8-2573-4f60-bf87-df447d57ab7a</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -21752,7 +21748,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Bute Inlet Geohazard - Topography Surveys - 2023 - Hakai Airborne Coastal Observatory</t>
+          <t>USGS Glacier Mapping - 2023 - Hakai Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -21794,16 +21790,16 @@
         </is>
       </c>
       <c r="N195" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.9, 50.53], [-124.2, 50.53], [-124.2, 50.99], [-124.9, 50.99], [-124.9, 50.53]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.4, 47.68], [-113.0, 47.68], [-113.0, 49.08], [-121.4, 49.08], [-121.4, 47.68]]]}</t>
         </is>
       </c>
       <c r="P195" t="inlineStr">
         <is>
-          <t>[{'max': '2600.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2800.0', 'min': '100.0'}]</t>
         </is>
       </c>
       <c r="Q195" t="inlineStr">
@@ -21813,12 +21809,12 @@
       </c>
       <c r="R195" t="inlineStr">
         <is>
-          <t>10.21966/e4b8-vp48</t>
+          <t>10.21966/bzr6-er66</t>
         </is>
       </c>
       <c r="S195" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRG7xQ84LQrgS4jhie</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRKhzLRiCcp6ENuX2r</t>
         </is>
       </c>
       <c r="T195" t="inlineStr">
@@ -21828,15 +21824,15 @@
       </c>
       <c r="U195" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V195" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W195" t="inlineStr">
         <is>
-          <t>[{'year': '2026', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X195" t="inlineStr"/>
@@ -21847,12 +21843,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>ca-cioos_43422dc8-2573-4f60-bf87-df447d57ab7a</t>
+          <t>ca-cioos_33a367c1-2706-4301-af99-4455fbe189a0</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -21862,7 +21858,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>USGS Glacier Mapping - 2023 - Hakai Airborne Coastal Observatory</t>
+          <t>Cryosphere Snow Surveys Southwest British Columbia - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -21908,12 +21904,12 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.4, 47.68], [-113.0, 47.68], [-113.0, 49.08], [-121.4, 49.08], [-121.4, 47.68]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.9, 48.62], [-122.1, 48.62], [-122.1, 50.82], [-126.9, 50.82], [-126.9, 48.62]]]}</t>
         </is>
       </c>
       <c r="P196" t="inlineStr">
         <is>
-          <t>[{'max': '2800.0', 'min': '100.0'}]</t>
+          <t>[{'max': '2300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q196" t="inlineStr">
@@ -21923,12 +21919,12 @@
       </c>
       <c r="R196" t="inlineStr">
         <is>
-          <t>10.21966/bzr6-er66</t>
+          <t>10.21966/thq7-0g08</t>
         </is>
       </c>
       <c r="S196" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRKhzLRiCcp6ENuX2r</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRfMcU9I8mMcBH6qiv</t>
         </is>
       </c>
       <c r="T196" t="inlineStr">
@@ -21938,7 +21934,7 @@
       </c>
       <c r="U196" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V196" t="n">
@@ -21949,7 +21945,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X196" t="inlineStr"/>
+      <c r="X196" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -30968,7 +30966,7 @@
         </is>
       </c>
       <c r="X278" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="279">
@@ -31199,12 +31197,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
+          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -31214,17 +31212,17 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
+          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>collection</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H281" t="b">
@@ -31237,7 +31235,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -31260,27 +31258,23 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
         </is>
       </c>
       <c r="P281" t="inlineStr">
         <is>
-          <t>[{'max': '2.5', 'min': '2.5'}]</t>
+          <t>[{'max': '0.0', 'min': '600.0'}]</t>
         </is>
       </c>
       <c r="Q281" t="inlineStr">
         <is>
-          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R281" t="inlineStr">
-        <is>
-          <t>10.21966/rrzq-yw32</t>
-        </is>
-      </c>
+          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R281" t="inlineStr"/>
       <c r="S281" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
         </is>
       </c>
       <c r="T281" t="inlineStr">
@@ -31293,15 +31287,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="V281" t="n">
-        <v>0</v>
-      </c>
-      <c r="W281" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X281" t="inlineStr"/>
+      <c r="V281" t="inlineStr"/>
+      <c r="W281" t="inlineStr"/>
+      <c r="X281" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="n">
@@ -31309,12 +31299,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
+          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -31324,17 +31314,17 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
+          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>collection</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H282" t="b">
@@ -31347,7 +31337,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -31370,23 +31360,27 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
         </is>
       </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '600.0'}]</t>
+          <t>[{'max': '2.5', 'min': '2.5'}]</t>
         </is>
       </c>
       <c r="Q282" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R282" t="inlineStr"/>
+          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr">
+        <is>
+          <t>10.21966/rrzq-yw32</t>
+        </is>
+      </c>
       <c r="S282" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
         </is>
       </c>
       <c r="T282" t="inlineStr">
@@ -31399,10 +31393,16 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="V282" t="inlineStr"/>
-      <c r="W282" t="inlineStr"/>
+      <c r="V282" t="n">
+        <v>0</v>
+      </c>
+      <c r="W282" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="X282" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="283">
@@ -31411,12 +31411,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
+          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>ca-cioos_bea3da72-dafe-4e25-b5b2-0176e0ffba44</t>
+          <t>ca-cioos_05c75bd9-1953-4ab9-8573-878845854662</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -31426,7 +31426,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Chemainus River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Glendale River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -31472,7 +31472,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.66843, 48.91641], [-123.6484, 48.90105], [-123.6554, 48.88016], [-123.6751, 48.87641], [-123.68894, 48.88178], [-123.68329, 48.89633], [-123.67928, 48.90316], [-123.67136, 48.91722], [-123.66848, 48.91635]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.72874, 50.69623], [-125.7357, 50.67697], [-125.73637, 50.66065], [-125.72893, 50.65255], [-125.71434, 50.64835], [-125.71329, 50.65188], [-125.72626, 50.65827], [-125.72636, 50.66466], [-125.72865, 50.68116], [-125.72721, 50.69604], [-125.72855, 50.69614], [-125.72874, 50.69623]]]}</t>
         </is>
       </c>
       <c r="P283" t="inlineStr">
@@ -31487,12 +31487,12 @@
       </c>
       <c r="R283" t="inlineStr">
         <is>
-          <t>10.21966/q2e0-j004</t>
+          <t>10.21966/r9zr-xz33</t>
         </is>
       </c>
       <c r="S283" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpszvIrt9OF8-BLQW2N</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7FmsNQ6HChfyLfTcX</t>
         </is>
       </c>
       <c r="T283" t="inlineStr">
@@ -31502,7 +31502,7 @@
       </c>
       <c r="U283" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="V283" t="n">
@@ -31514,7 +31514,7 @@
         </is>
       </c>
       <c r="X283" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="284">
@@ -31523,12 +31523,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+          <t>c428c9ff-19ed-40ec-82e0-40ab10960364</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+          <t>ca-cioos_0e50f5a3-6100-4f1a-b184-ba327def9f3a</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -31538,7 +31538,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kaouk River estuary (Provisional)</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -31556,12 +31556,12 @@
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Estuary Resilience</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -31576,7 +31576,7 @@
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>Tula Foundation</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N284" t="n">
@@ -31584,44 +31584,1836 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.15825, 50.07693], [-127.15157, 50.07806], [-127.13204, 50.06944], [-127.11152, 50.06781], [-127.0959, 50.06667], [-127.04315, 50.06879], [-127.04168, 50.06455], [-127.0902, 50.05983], [-127.10062, 50.05658], [-127.11983, 50.05885], [-127.13887, 50.06423], [-127.15988, 50.0753], [-127.15874, 50.07693], [-127.15825, 50.07693]]]}</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R284" t="inlineStr">
+        <is>
+          <t>10.21966/9dbb-5d54</t>
+        </is>
+      </c>
+      <c r="S284" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq6X1wQRkybrW6sac5D</t>
+        </is>
+      </c>
+      <c r="T284" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U284" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V284" t="n">
+        <v>0</v>
+      </c>
+      <c r="W284" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X284" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>283</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>ca-cioos_2ba57f02-c88b-42b8-8f8c-07cfdeab45d3</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Kw'a'luxw River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H285" t="b">
+        <v>0</v>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N285" t="n">
+        <v>1</v>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.29886, 49.3576], [-124.30659, 49.32057], [-124.28624, 49.31332], [-124.26557, 49.29566], [-124.26427, 49.29899], [-124.28624, 49.3283], [-124.29878, 49.35744], [-124.29886, 49.3576]]]}</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R285" t="inlineStr">
+        <is>
+          <t>10.21966/vpz7-mm73</t>
+        </is>
+      </c>
+      <c r="S285" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptH1k-7T2gjAKY814I</t>
+        </is>
+      </c>
+      <c r="T285" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U285" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V285" t="n">
+        <v>0</v>
+      </c>
+      <c r="W285" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X285" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>284</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>0ce3ee5b-425b-4eb0-a201-96bdfb795a3f</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>ca-cioos_354b5b83-e752-4ffb-a740-d1cdc02ac8c6</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Dtlaxsiwè River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H286" t="b">
+        <v>0</v>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N286" t="n">
+        <v>1</v>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.1721, 50.61011], [-127.17933, 50.612], [-127.1873, 50.6098], [-127.19703, 50.61072], [-127.20524, 50.61585], [-127.19007, 50.61844], [-127.18675, 50.61393], [-127.17744, 50.61359], [-127.17161, 50.61118], [-127.17203, 50.61011], [-127.1721, 50.61011]]]}</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R286" t="inlineStr">
+        <is>
+          <t>10.21966/ydm2-m238</t>
+        </is>
+      </c>
+      <c r="S286" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7Dng-ZtRd05hnZCq1</t>
+        </is>
+      </c>
+      <c r="T286" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U286" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V286" t="n">
+        <v>0</v>
+      </c>
+      <c r="W286" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X286" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>285</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1a2aa5c8-9a83-46f7-967d-1127436c2084</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>ca-cioos_58a5140a-0b2c-4186-a648-53d9f58e5226</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Kvai River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H287" t="b">
+        <v>0</v>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N287" t="n">
+        <v>1</v>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.81882, 51.77547], [-127.83122, 51.77986], [-127.85192, 51.781], [-127.86785, 51.78358], [-127.8958, 51.77366], [-127.89418, 51.77118], [-127.87834, 51.77309], [-127.86508, 51.77748], [-127.84009, 51.77519], [-127.82731, 51.77452], [-127.82025, 51.77309], [-127.81853, 51.77566], [-127.81882, 51.77547]]]}</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R287" t="inlineStr">
+        <is>
+          <t>10.21966/pm9m-h431</t>
+        </is>
+      </c>
+      <c r="S287" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7QQE3ifLCAPcu3Jih</t>
+        </is>
+      </c>
+      <c r="T287" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U287" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V287" t="n">
+        <v>0</v>
+      </c>
+      <c r="W287" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X287" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>286</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>c035b81c-0fc3-446e-bec5-8b8933ae874b</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>ca-cioos_7fbc28f7-ee87-4361-bbee-0ed8ce24522d</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Gwa'dzi River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H288" t="b">
+        <v>0</v>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N288" t="n">
+        <v>1</v>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.46176, 50.74217], [-127.49022, 50.72165], [-127.49167, 50.71188], [-127.4832, 50.70356], [-127.4874, 50.69181], [-127.46443, 50.6928], [-127.47282, 50.70776], [-127.47992, 50.71424], [-127.48305, 50.72058], [-127.45901, 50.74011], [-127.46153, 50.74217], [-127.46176, 50.74217]]]}</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R288" t="inlineStr">
+        <is>
+          <t>10.21966/xq99-x273</t>
+        </is>
+      </c>
+      <c r="S288" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7BCRnF2C30YPkxIyd</t>
+        </is>
+      </c>
+      <c r="T288" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U288" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V288" t="n">
+        <v>0</v>
+      </c>
+      <c r="W288" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X288" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>287</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H289" t="b">
+        <v>0</v>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N289" t="n">
+        <v>1</v>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R289" t="inlineStr">
+        <is>
+          <t>10.21966/kde9-8g12</t>
+        </is>
+      </c>
+      <c r="S289" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
+        </is>
+      </c>
+      <c r="T289" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U289" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V289" t="n">
+        <v>0</v>
+      </c>
+      <c r="W289" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X289" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>288</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H290" t="b">
+        <v>0</v>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N290" t="n">
+        <v>1</v>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R290" t="inlineStr">
+        <is>
+          <t>10.21966/9a97-2j48</t>
+        </is>
+      </c>
+      <c r="S290" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
+        </is>
+      </c>
+      <c r="T290" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U290" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V290" t="n">
+        <v>0</v>
+      </c>
+      <c r="W290" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X290" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>289</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>ca-cioos_86f1dd95-27a0-4c52-97e4-15be649ce73a</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Xwésam River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H291" t="b">
+        <v>0</v>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N291" t="n">
+        <v>1</v>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.92043, 50.31848], [-125.94107, 50.31848], [-125.94046, 50.36243], [-125.9639, 50.38185], [-125.95731, 50.39906], [-125.94094, 50.38954], [-125.93716, 50.37831], [-125.91445, 50.37257], [-125.91994, 50.31835], [-125.92043, 50.31848]]]}</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R291" t="inlineStr">
+        <is>
+          <t>10.21966/ed9w-2653</t>
+        </is>
+      </c>
+      <c r="S291" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptUCw9y_sktWpuppc0</t>
+        </is>
+      </c>
+      <c r="T291" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U291" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V291" t="n">
+        <v>0</v>
+      </c>
+      <c r="W291" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X291" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>290</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>1af6a43a-e73b-4774-8e10-b9f2928ab133</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>ca-cioos_ae7e017c-9211-4f98-b56e-90a4bbac161c</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Snuneymuxw River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H292" t="b">
+        <v>0</v>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N292" t="n">
+        <v>1</v>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.88685, 49.19332], [-123.92494, 49.1612], [-123.92581, 49.13841], [-123.91159, 49.123], [-123.88023, 49.11117], [-123.85971, 49.12766], [-123.89792, 49.16196], [-123.88099, 49.18866], [-123.88685, 49.19332]]]}</t>
+        </is>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R292" t="inlineStr">
+        <is>
+          <t>10.21966/k01q-wb27</t>
+        </is>
+      </c>
+      <c r="S292" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt459vxCIH7YPRN9fp</t>
+        </is>
+      </c>
+      <c r="T292" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U292" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V292" t="n">
+        <v>0</v>
+      </c>
+      <c r="W292" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X292" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>291</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>d320d90e-96bf-4993-81c5-f1f57886b0e6</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>ca-cioos_b922699f-69b6-4d63-b538-7c290086a408</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Quw'utsun/Xwulqw'selu River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H293" t="b">
+        <v>0</v>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N293" t="n">
+        <v>1</v>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.56201, 48.73508], [-123.59772, 48.75559], [-123.62127, 48.76514], [-123.63885, 48.77426], [-123.66935, 48.78033], [-123.67901, 48.75472], [-123.65155, 48.74322], [-123.63017, 48.7405], [-123.60792, 48.74289], [-123.56494, 48.72987], [-123.56179, 48.73529], [-123.56201, 48.73508]]]}</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R293" t="inlineStr">
+        <is>
+          <t>10.21966/2ha7-9p26</t>
+        </is>
+      </c>
+      <c r="S293" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpsCA3ycwZ7bFTDIQxh</t>
+        </is>
+      </c>
+      <c r="T293" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U293" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V293" t="n">
+        <v>0</v>
+      </c>
+      <c r="W293" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X293" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>292</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>ca-cioos_bea3da72-dafe-4e25-b5b2-0176e0ffba44</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Chemainus River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H294" t="b">
+        <v>0</v>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N294" t="n">
+        <v>1</v>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.66843, 48.91641], [-123.6484, 48.90105], [-123.6554, 48.88016], [-123.6751, 48.87641], [-123.68894, 48.88178], [-123.68329, 48.89633], [-123.67928, 48.90316], [-123.67136, 48.91722], [-123.66848, 48.91635], [-123.66843, 48.91641]]]}</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R294" t="inlineStr">
+        <is>
+          <t>10.21966/q2e0-j004</t>
+        </is>
+      </c>
+      <c r="S294" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpszvIrt9OF8-BLQW2N</t>
+        </is>
+      </c>
+      <c r="T294" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U294" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V294" t="n">
+        <v>0</v>
+      </c>
+      <c r="W294" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X294" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>293</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H295" t="b">
+        <v>0</v>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N295" t="n">
+        <v>1</v>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
+        </is>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R295" t="inlineStr">
+        <is>
+          <t>10.21966/hjkj-6611</t>
+        </is>
+      </c>
+      <c r="S295" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
+        </is>
+      </c>
+      <c r="T295" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U295" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V295" t="n">
+        <v>0</v>
+      </c>
+      <c r="W295" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X295" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>294</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>4c7b7347-767d-45e4-b3ad-7e0133b31e1c</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>ca-cioos_dce15b7b-3772-4106-ab20-c3979c4c3f57</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Fulmore River - Shoal Creek Estuary Complex (Provisional)</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H296" t="b">
+        <v>0</v>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N296" t="n">
+        <v>1</v>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.08798, 50.4777], [-126.09599, 50.48418], [-126.09046, 50.50918], [-126.0647, 50.52425], [-125.99698, 50.53569], [-125.93459, 50.56717], [-125.93173, 50.56202], [-125.93764, 50.55458], [-125.91055, 50.55134], [-125.89853, 50.54943], [-125.90063, 50.54466], [-125.96416, 50.53989], [-125.98973, 50.52043], [-126.06566, 50.5067], [-126.08779, 50.47789], [-126.08798, 50.4777]]]}</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R296" t="inlineStr">
+        <is>
+          <t>10.21966/g1cn-xs92</t>
+        </is>
+      </c>
+      <c r="S296" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptdJ8iUmLeOrdmqzrQ</t>
+        </is>
+      </c>
+      <c r="T296" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U296" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V296" t="n">
+        <v>0</v>
+      </c>
+      <c r="W296" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X296" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>295</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H297" t="b">
+        <v>0</v>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N297" t="n">
+        <v>1</v>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
+        </is>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R297" t="inlineStr">
+        <is>
+          <t>10.21966/npe4-3036</t>
+        </is>
+      </c>
+      <c r="S297" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
+        </is>
+      </c>
+      <c r="T297" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U297" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V297" t="n">
+        <v>0</v>
+      </c>
+      <c r="W297" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X297" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>296</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>35245eae-e508-47da-bcf7-54346cda086a</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>ca-cioos_e9b72149-8cf1-4000-ae3e-6b29ad60b078</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Malksope River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H298" t="b">
+        <v>0</v>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N298" t="n">
+        <v>1</v>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.46569, 50.12556], [-127.45723, 50.13142], [-127.43281, 50.13338], [-127.42845, 50.13765], [-127.41181, 50.14408], [-127.40973, 50.14233], [-127.41999, 50.13627], [-127.41803, 50.13195], [-127.43106, 50.12796], [-127.46545, 50.12446], [-127.46569, 50.12548], [-127.46569, 50.12556]]]}</t>
+        </is>
+      </c>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R298" t="inlineStr">
+        <is>
+          <t>10.21966/21sf-ey03</t>
+        </is>
+      </c>
+      <c r="S298" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq77iyWJfPg4z-FvOSb</t>
+        </is>
+      </c>
+      <c r="T298" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U298" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V298" t="n">
+        <v>0</v>
+      </c>
+      <c r="W298" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X298" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>297</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>5177d019-598e-4415-b778-9688403652c8</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>ca-cioos_ed84df74-5a2d-4a7d-87c8-a7b93f11088e</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Nalaxdlala River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H299" t="b">
+        <v>0</v>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N299" t="n">
+        <v>1</v>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.9489, 50.70902], [-125.9696, 50.70291], [-126.00938, 50.69118], [-126.00108, 50.66848], [-125.98257, 50.68374], [-125.98152, 50.69271], [-125.95462, 50.70263], [-125.94785, 50.70768], [-125.9489, 50.70911], [-125.9489, 50.70902]]]}</t>
+        </is>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R299" t="inlineStr">
+        <is>
+          <t>10.21966/4krv-aw23</t>
+        </is>
+      </c>
+      <c r="S299" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptbxmpkBsfyWWfSxOJ</t>
+        </is>
+      </c>
+      <c r="T299" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U299" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V299" t="n">
+        <v>0</v>
+      </c>
+      <c r="W299" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X299" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>298</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H300" t="b">
+        <v>0</v>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory, Geospatial</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>Tula Foundation</t>
+        </is>
+      </c>
+      <c r="N300" t="n">
+        <v>1</v>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
           <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
         </is>
       </c>
-      <c r="P284" t="inlineStr">
+      <c r="P300" t="inlineStr">
         <is>
           <t>[{'max': '3954.0', 'min': '800.0'}]</t>
         </is>
       </c>
-      <c r="Q284" t="inlineStr">
+      <c r="Q300" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="R284" t="inlineStr">
+      <c r="R300" t="inlineStr">
         <is>
           <t>10.21966/w9n0-kn30</t>
         </is>
       </c>
-      <c r="S284" t="inlineStr">
+      <c r="S300" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
         </is>
       </c>
-      <c r="T284" t="inlineStr"/>
-      <c r="U284" t="inlineStr">
+      <c r="T300" t="inlineStr"/>
+      <c r="U300" t="inlineStr">
         <is>
           <t>2025-04-02</t>
         </is>
       </c>
-      <c r="V284" t="n">
-        <v>0</v>
-      </c>
-      <c r="W284" t="inlineStr">
+      <c r="V300" t="n">
+        <v>0</v>
+      </c>
+      <c r="W300" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="X284" t="inlineStr"/>
+      <c r="X300" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>